<commit_message>
update README, split out some into docs/
</commit_message>
<xml_diff>
--- a/examples/all_features.xlsx
+++ b/examples/all_features.xlsx
@@ -11,7 +11,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mv="urn:schemas-microsoft-com:mac:vml">
   <numFmts count="0"/>
-  <fonts count="138">
+  <fonts count="146">
     <font>
       <name val="Verdana"/>
       <sz val="10"/>
@@ -60,6 +60,50 @@
     <font>
       <name val="Verdana"/>
       <sz val="20"/>
+    </font>
+    <font>
+      <name val="Verdana"/>
+      <b val="1"/>
+      <sz val="10"/>
+      <u val="1"/>
+    </font>
+    <font>
+      <name val="Verdana"/>
+      <sz val="10"/>
+      <u val="1"/>
+    </font>
+    <font>
+      <name val="Verdana"/>
+      <b val="1"/>
+      <sz val="10"/>
+      <u val="1"/>
+    </font>
+    <font>
+      <name val="Verdana"/>
+      <sz val="10"/>
+      <u val="1"/>
+    </font>
+    <font>
+      <name val="Verdana"/>
+      <b val="1"/>
+      <sz val="10"/>
+      <u val="1"/>
+    </font>
+    <font>
+      <name val="Verdana"/>
+      <sz val="10"/>
+      <u val="1"/>
+    </font>
+    <font>
+      <name val="Verdana"/>
+      <b val="1"/>
+      <sz val="10"/>
+      <u val="1"/>
+    </font>
+    <font>
+      <name val="Verdana"/>
+      <sz val="10"/>
+      <u val="1"/>
     </font>
     <font>
       <name val="Verdana"/>
@@ -906,7 +950,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="188">
+  <cellXfs count="196">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1387,6 +1431,30 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="137" fillId="0" borderId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="138" fillId="0" borderId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="139" fillId="0" borderId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="140" fillId="0" borderId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="141" fillId="0" borderId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="142" fillId="0" borderId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="143" fillId="0" borderId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="144" fillId="0" borderId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="145" fillId="0" borderId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1722,7 +1790,7 @@
       <c r="A1" s="57" t="str">
         <v>Header1</v>
       </c>
-      <c r="B1" s="186" t="str">
+      <c r="B1" s="194" t="str">
         <v>Header2</v>
       </c>
       <c r="C1" s="62" t="str">
@@ -1739,7 +1807,7 @@
       <c r="A2" s="12" t="str">
         <v>=ADD(1, 2)</v>
       </c>
-      <c r="B2" s="187" t="str">
+      <c r="B2" s="195" t="str">
         <v>=1</v>
       </c>
       <c r="C2" s="12" t="str">

</xml_diff>